<commit_message>
ajout Observations, mapping, exmeples 7bb7923fdd05fd06d6ae3ea7cb240ffcbf02ea8b
</commit_message>
<xml_diff>
--- a/417-contenu-fhir---ajout-des-causes-de-décès/ig/CodeSystem-tddui-observation-periode-scolaire.xlsx
+++ b/417-contenu-fhir---ajout-des-causes-de-décès/ig/CodeSystem-tddui-observation-periode-scolaire.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-02-06T10:49:33+00:00</t>
+    <t>2026-02-10T10:00:25+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -156,7 +156,7 @@
     <t>typeEnseignementSpecialise</t>
   </si>
   <si>
-    <t>Type d'enseignement spécialisé</t>
+    <t>Type enseignement spécialisé</t>
   </si>
   <si>
     <t>diplome</t>

</xml_diff>